<commit_message>
suspense 2nd and 4th
edit suspense for 2nd and 4th battle, wc 2018 D minute 76
</commit_message>
<xml_diff>
--- a/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
+++ b/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
@@ -678,7 +678,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'France', 'Hungary']</t>
+          <t>['Hungary', 'France', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -2854,7 +2854,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>['Belgium', 'Mexico', 'Paraguay']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>['Belgium', 'Mexico', 'Paraguay']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>['Belgium', 'Mexico', 'Paraguay']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>['Belgium', 'Mexico', 'Paraguay']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>['Mexico', 'Paraguay', 'Belgium']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>['Belgium', 'Mexico', 'Paraguay']</t>
+          <t>['Paraguay', 'Mexico', 'Belgium']</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -3784,7 +3784,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>['Morocco', 'Portugal', 'Poland']</t>
+          <t>['Portugal', 'Poland', 'Morocco']</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>['Portugal', 'England', 'Poland']</t>
+          <t>['Portugal', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>['Morocco', 'Portugal', 'England']</t>
+          <t>['Portugal', 'England', 'Morocco']</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>['Morocco', 'England', 'Poland']</t>
+          <t>['Morocco', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>['Morocco', 'England', 'Poland']</t>
+          <t>['Morocco', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>['Morocco', 'England', 'Poland']</t>
+          <t>['Morocco', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>['Morocco', 'England', 'Poland']</t>
+          <t>['Morocco', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>['Morocco', 'England', 'Poland']</t>
+          <t>['Morocco', 'Poland', 'England']</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -5030,7 +5030,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>['Brazil', 'Spain', 'Algeria']</t>
+          <t>['Algeria', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>['Brazil', 'Spain', 'Algeria']</t>
+          <t>['Algeria', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -6118,7 +6118,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>['Denmark', 'West Germany', 'Uruguay']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>['Denmark', 'West Germany', 'Uruguay']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>['Denmark', 'West Germany', 'Uruguay']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -6574,7 +6574,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Cameroon', 'Argentina']</t>
+          <t>['Argentina', 'Cameroon', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Argentina', 'Romania']</t>
+          <t>['Romania', 'Argentina', 'Cameroon']</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -7662,7 +7662,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Colombia', 'West Germany']</t>
+          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -8908,7 +8908,7 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -9694,7 +9694,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>['Italy', 'Czechoslovakia', 'Austria']</t>
+          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -9838,7 +9838,7 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>['Scotland', 'Brazil', 'Costa Rica']</t>
+          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>['Sweden', 'Scotland', 'Brazil']</t>
+          <t>['Scotland', 'Sweden', 'Brazil']</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>['Scotland', 'Brazil', 'Costa Rica']</t>
+          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>['Scotland', 'Brazil', 'Costa Rica']</t>
+          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>['Scotland', 'Brazil', 'Costa Rica']</t>
+          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -10610,7 +10610,7 @@
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
-          <t>['Belgium', 'Spain', 'Uruguay']</t>
+          <t>['Uruguay', 'Belgium', 'Spain']</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>['Belgium', 'Spain', 'Uruguay']</t>
+          <t>['Uruguay', 'Belgium', 'Spain']</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>['Belgium', 'Spain', 'Uruguay']</t>
+          <t>['Uruguay', 'Belgium', 'Spain']</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>['Belgium', 'Spain', 'Uruguay']</t>
+          <t>['Uruguay', 'Belgium', 'Spain']</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>['Belgium', 'Spain', 'Uruguay']</t>
+          <t>['Uruguay', 'Belgium', 'Spain']</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -11382,7 +11382,7 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>['Ireland', 'Netherlands', 'England']</t>
+          <t>['Ireland', 'England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>['Egypt', 'Netherlands', 'England']</t>
+          <t>['Egypt', 'England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>['Egypt', 'Netherlands', 'England']</t>
+          <t>['Egypt', 'England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>['Ireland', 'Netherlands', 'England']</t>
+          <t>['Ireland', 'England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -11996,7 +11996,7 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['Switzerland', 'Romania', 'United States']</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -12150,7 +12150,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['Switzerland', 'Romania', 'United States']</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['Switzerland', 'Romania', 'United States']</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['Switzerland', 'Romania', 'United States']</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -12610,7 +12610,7 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -12922,7 +12922,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -13870,7 +13870,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany', 'South Korea']</t>
+          <t>['South Korea', 'Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>['Ireland', 'Italy', 'Norway']</t>
+          <t>['Italy', 'Norway', 'Ireland']</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -14782,7 +14782,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -15098,7 +15098,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -16046,7 +16046,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>['Sweden', 'Brazil', 'Russia']</t>
+          <t>['Sweden', 'Russia', 'Brazil']</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -17734,7 +17734,7 @@
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -17888,7 +17888,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -18046,7 +18046,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -18204,7 +18204,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -18362,7 +18362,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -18520,7 +18520,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>['Italy', 'Chile']</t>
+          <t>['Chile', 'Italy']</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -18664,7 +18664,7 @@
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
-          <t>['Brazil', 'Norway']</t>
+          <t>['Norway', 'Brazil']</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>['Brazil', 'Norway']</t>
+          <t>['Norway', 'Brazil']</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -26122,7 +26122,7 @@
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
-          <t>['Denmark', 'Senegal']</t>
+          <t>['Senegal', 'Denmark']</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -26434,7 +26434,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>['Denmark', 'Senegal']</t>
+          <t>['Senegal', 'Denmark']</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -27224,7 +27224,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>['Denmark', 'Senegal']</t>
+          <t>['Senegal', 'Denmark']</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>['Denmark', 'Senegal']</t>
+          <t>['Senegal', 'Denmark']</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -28912,7 +28912,7 @@
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -29066,7 +29066,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -29224,7 +29224,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -29382,7 +29382,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -29540,7 +29540,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -29698,7 +29698,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -29856,7 +29856,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -30014,7 +30014,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -30172,7 +30172,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -30330,7 +30330,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>['Spain', 'Paraguay']</t>
+          <t>['Paraguay', 'Spain']</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -30474,7 +30474,7 @@
       <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr">
         <is>
-          <t>['Brazil', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -30628,7 +30628,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>['Brazil', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -30786,7 +30786,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>['Brazil', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -30944,7 +30944,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -31102,7 +31102,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -31260,7 +31260,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -31418,7 +31418,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -31576,7 +31576,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>['Brazil', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Brazil']</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -31734,7 +31734,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -31892,7 +31892,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -32050,7 +32050,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>['Brazil', 'Turkey']</t>
+          <t>['Turkey', 'Brazil']</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -32194,7 +32194,7 @@
       <c r="I205" t="inlineStr"/>
       <c r="J205" t="inlineStr">
         <is>
-          <t>['Mexico', 'Italy']</t>
+          <t>['Italy', 'Mexico']</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -32348,7 +32348,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>['Mexico', 'Croatia']</t>
+          <t>['Croatia', 'Mexico']</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -32506,7 +32506,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>['Mexico', 'Italy']</t>
+          <t>['Italy', 'Mexico']</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -32664,7 +32664,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>['Mexico', 'Italy']</t>
+          <t>['Italy', 'Mexico']</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -32808,7 +32808,7 @@
       <c r="I209" t="inlineStr"/>
       <c r="J209" t="inlineStr">
         <is>
-          <t>['Japan', 'Russia']</t>
+          <t>['Russia', 'Japan']</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>['Japan', 'Belgium']</t>
+          <t>['Belgium', 'Japan']</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -33120,7 +33120,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>['Japan', 'Belgium']</t>
+          <t>['Belgium', 'Japan']</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -33278,7 +33278,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>['Japan', 'Russia']</t>
+          <t>['Russia', 'Japan']</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -33436,7 +33436,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>['Japan', 'Russia']</t>
+          <t>['Russia', 'Japan']</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -33594,7 +33594,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>['Japan', 'Belgium']</t>
+          <t>['Belgium', 'Japan']</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -33752,7 +33752,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>['Japan', 'Belgium']</t>
+          <t>['Belgium', 'Japan']</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>['Japan', 'Belgium']</t>
+          <t>['Belgium', 'Japan']</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -34054,7 +34054,7 @@
       <c r="I217" t="inlineStr"/>
       <c r="J217" t="inlineStr">
         <is>
-          <t>['United States', 'South Korea']</t>
+          <t>['South Korea', 'United States']</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -34208,7 +34208,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>['Portugal', 'South Korea']</t>
+          <t>['South Korea', 'Portugal']</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -34366,7 +34366,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>['Portugal', 'South Korea']</t>
+          <t>['South Korea', 'Portugal']</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>['Portugal', 'South Korea']</t>
+          <t>['South Korea', 'Portugal']</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -34682,7 +34682,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>['United States', 'South Korea']</t>
+          <t>['South Korea', 'United States']</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -34840,7 +34840,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>['United States', 'South Korea']</t>
+          <t>['South Korea', 'United States']</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -38090,7 +38090,7 @@
       <c r="I243" t="inlineStr"/>
       <c r="J243" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -38244,7 +38244,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -38402,7 +38402,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -38560,7 +38560,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -38718,7 +38718,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -38876,7 +38876,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -39174,7 +39174,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>['Ghana', 'Italy']</t>
+          <t>['Italy', 'Ghana']</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -39332,7 +39332,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>['Ghana', 'Italy']</t>
+          <t>['Italy', 'Ghana']</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -39490,7 +39490,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>['Ghana', 'Italy']</t>
+          <t>['Italy', 'Ghana']</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -39648,7 +39648,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>['Ghana', 'Italy']</t>
+          <t>['Italy', 'Ghana']</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -39806,7 +39806,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>['Ghana', 'Italy']</t>
+          <t>['Italy', 'Ghana']</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -39950,7 +39950,7 @@
       <c r="I255" t="inlineStr"/>
       <c r="J255" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -40420,7 +40420,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -40578,7 +40578,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -40736,7 +40736,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -41210,7 +41210,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -41368,7 +41368,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>['Brazil', 'Australia']</t>
+          <t>['Australia', 'Brazil']</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -41512,7 +41512,7 @@
       <c r="I265" t="inlineStr"/>
       <c r="J265" t="inlineStr">
         <is>
-          <t>['Spain', 'Ukraine']</t>
+          <t>['Ukraine', 'Spain']</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -41666,7 +41666,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>['Spain', 'Ukraine']</t>
+          <t>['Ukraine', 'Spain']</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -41824,7 +41824,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>['Spain', 'Ukraine']</t>
+          <t>['Ukraine', 'Spain']</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -42280,7 +42280,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -42438,7 +42438,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -42596,7 +42596,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -42740,7 +42740,7 @@
       <c r="I273" t="inlineStr"/>
       <c r="J273" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -42894,7 +42894,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -43052,7 +43052,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -43210,7 +43210,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -43368,7 +43368,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -43666,7 +43666,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>['Greece', 'Argentina']</t>
+          <t>['Argentina', 'Greece']</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -44912,7 +44912,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>['United States', 'England']</t>
+          <t>['England', 'United States']</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -45982,7 +45982,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Paraguay']</t>
+          <t>['Paraguay', 'Slovakia']</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -46140,7 +46140,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Paraguay']</t>
+          <t>['Paraguay', 'Slovakia']</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -46298,7 +46298,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Paraguay']</t>
+          <t>['Paraguay', 'Slovakia']</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -46456,7 +46456,7 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Paraguay']</t>
+          <t>['Paraguay', 'Slovakia']</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
@@ -46614,7 +46614,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Paraguay']</t>
+          <t>['Paraguay', 'Slovakia']</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -48618,7 +48618,7 @@
       <c r="I311" t="inlineStr"/>
       <c r="J311" t="inlineStr">
         <is>
-          <t>['Spain', 'Chile']</t>
+          <t>['Chile', 'Spain']</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -48772,7 +48772,7 @@
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>['Spain', 'Chile']</t>
+          <t>['Chile', 'Spain']</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
@@ -48930,7 +48930,7 @@
       </c>
       <c r="J313" t="inlineStr">
         <is>
-          <t>['Spain', 'Chile']</t>
+          <t>['Chile', 'Spain']</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
@@ -49088,7 +49088,7 @@
       </c>
       <c r="J314" t="inlineStr">
         <is>
-          <t>['Spain', 'Chile']</t>
+          <t>['Chile', 'Spain']</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
@@ -49232,7 +49232,7 @@
       <c r="I315" t="inlineStr"/>
       <c r="J315" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -49386,7 +49386,7 @@
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -49544,7 +49544,7 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -49702,7 +49702,7 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -49860,7 +49860,7 @@
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -50018,7 +50018,7 @@
       </c>
       <c r="J320" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Chile']</t>
+          <t>['Chile', 'Netherlands']</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
@@ -51724,7 +51724,7 @@
       <c r="I331" t="inlineStr"/>
       <c r="J331" t="inlineStr">
         <is>
-          <t>['Italy', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Italy']</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
@@ -51878,7 +51878,7 @@
       </c>
       <c r="J332" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Uruguay']</t>
+          <t>['Uruguay', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K332" t="inlineStr">
@@ -52022,7 +52022,7 @@
       <c r="I333" t="inlineStr"/>
       <c r="J333" t="inlineStr">
         <is>
-          <t>['Colombia', 'Ivory Coast']</t>
+          <t>['Ivory Coast', 'Colombia']</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">
@@ -52176,7 +52176,7 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>['Colombia', 'Ivory Coast']</t>
+          <t>['Ivory Coast', 'Colombia']</t>
         </is>
       </c>
       <c r="K334" t="inlineStr">
@@ -52334,7 +52334,7 @@
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
@@ -52492,7 +52492,7 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
@@ -52650,7 +52650,7 @@
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
@@ -52808,7 +52808,7 @@
       </c>
       <c r="J338" t="inlineStr">
         <is>
-          <t>['Colombia', 'Ivory Coast']</t>
+          <t>['Ivory Coast', 'Colombia']</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
@@ -52966,7 +52966,7 @@
       </c>
       <c r="J339" t="inlineStr">
         <is>
-          <t>['Colombia', 'Ivory Coast']</t>
+          <t>['Ivory Coast', 'Colombia']</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
@@ -53124,7 +53124,7 @@
       </c>
       <c r="J340" t="inlineStr">
         <is>
-          <t>['Colombia', 'Ivory Coast']</t>
+          <t>['Ivory Coast', 'Colombia']</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
@@ -53282,7 +53282,7 @@
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -54988,7 +54988,7 @@
       <c r="I352" t="inlineStr"/>
       <c r="J352" t="inlineStr">
         <is>
-          <t>['France', 'Ecuador']</t>
+          <t>['Ecuador', 'France']</t>
         </is>
       </c>
       <c r="K352" t="inlineStr">
@@ -55142,7 +55142,7 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
@@ -55300,7 +55300,7 @@
       </c>
       <c r="J354" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K354" t="inlineStr">
@@ -55458,7 +55458,7 @@
       </c>
       <c r="J355" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland']</t>
+          <t>['Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K355" t="inlineStr">
@@ -55602,7 +55602,7 @@
       <c r="I356" t="inlineStr"/>
       <c r="J356" t="inlineStr">
         <is>
-          <t>['United States', 'Germany']</t>
+          <t>['Germany', 'United States']</t>
         </is>
       </c>
       <c r="K356" t="inlineStr">
@@ -55756,7 +55756,7 @@
       </c>
       <c r="J357" t="inlineStr">
         <is>
-          <t>['United States', 'Germany']</t>
+          <t>['Germany', 'United States']</t>
         </is>
       </c>
       <c r="K357" t="inlineStr">
@@ -55914,7 +55914,7 @@
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>['United States', 'Germany']</t>
+          <t>['Germany', 'United States']</t>
         </is>
       </c>
       <c r="K358" t="inlineStr">
@@ -56072,7 +56072,7 @@
       </c>
       <c r="J359" t="inlineStr">
         <is>
-          <t>['United States', 'Germany']</t>
+          <t>['Germany', 'United States']</t>
         </is>
       </c>
       <c r="K359" t="inlineStr">
@@ -56230,7 +56230,7 @@
       </c>
       <c r="J360" t="inlineStr">
         <is>
-          <t>['United States', 'Germany']</t>
+          <t>['Germany', 'United States']</t>
         </is>
       </c>
       <c r="K360" t="inlineStr">
@@ -56374,7 +56374,7 @@
       <c r="I361" t="inlineStr"/>
       <c r="J361" t="inlineStr">
         <is>
-          <t>['Belgium', 'Algeria']</t>
+          <t>['Algeria', 'Belgium']</t>
         </is>
       </c>
       <c r="K361" t="inlineStr">
@@ -56528,7 +56528,7 @@
       </c>
       <c r="J362" t="inlineStr">
         <is>
-          <t>['Belgium', 'Russia']</t>
+          <t>['Russia', 'Belgium']</t>
         </is>
       </c>
       <c r="K362" t="inlineStr">
@@ -56686,7 +56686,7 @@
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>['Belgium', 'Algeria']</t>
+          <t>['Algeria', 'Belgium']</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
@@ -56844,7 +56844,7 @@
       </c>
       <c r="J364" t="inlineStr">
         <is>
-          <t>['Belgium', 'Algeria']</t>
+          <t>['Algeria', 'Belgium']</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
@@ -56988,7 +56988,7 @@
       <c r="I365" t="inlineStr"/>
       <c r="J365" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
@@ -57142,7 +57142,7 @@
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
@@ -57300,7 +57300,7 @@
       </c>
       <c r="J367" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K367" t="inlineStr">
@@ -57458,7 +57458,7 @@
       </c>
       <c r="J368" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K368" t="inlineStr">
@@ -57616,7 +57616,7 @@
       </c>
       <c r="J369" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K369" t="inlineStr">
@@ -57774,7 +57774,7 @@
       </c>
       <c r="J370" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K370" t="inlineStr">
@@ -57932,7 +57932,7 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -60361,7 +60361,7 @@
         <v>0</v>
       </c>
       <c r="AR386" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="387">
@@ -61638,7 +61638,7 @@
       <c r="I395" t="inlineStr"/>
       <c r="J395" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
@@ -61792,7 +61792,7 @@
       </c>
       <c r="J396" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
@@ -61950,7 +61950,7 @@
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
@@ -62108,7 +62108,7 @@
       </c>
       <c r="J398" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
@@ -62266,7 +62266,7 @@
       </c>
       <c r="J399" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
@@ -62424,7 +62424,7 @@
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
@@ -62582,7 +62582,7 @@
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
@@ -62726,7 +62726,7 @@
       <c r="I402" t="inlineStr"/>
       <c r="J402" t="inlineStr">
         <is>
-          <t>['Japan', 'Senegal']</t>
+          <t>['Senegal', 'Japan']</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
@@ -64884,7 +64884,7 @@
       <c r="I416" t="inlineStr"/>
       <c r="J416" t="inlineStr">
         <is>
-          <t>['England', 'Iran']</t>
+          <t>['Iran', 'England']</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
@@ -65038,7 +65038,7 @@
       </c>
       <c r="J417" t="inlineStr">
         <is>
-          <t>['United States', 'England']</t>
+          <t>['England', 'United States']</t>
         </is>
       </c>
       <c r="K417" t="inlineStr">
@@ -65196,7 +65196,7 @@
       </c>
       <c r="J418" t="inlineStr">
         <is>
-          <t>['United States', 'England']</t>
+          <t>['England', 'United States']</t>
         </is>
       </c>
       <c r="K418" t="inlineStr">
@@ -65354,7 +65354,7 @@
       </c>
       <c r="J419" t="inlineStr">
         <is>
-          <t>['United States', 'England']</t>
+          <t>['England', 'United States']</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="J420" t="inlineStr">
         <is>
-          <t>['United States', 'England']</t>
+          <t>['England', 'United States']</t>
         </is>
       </c>
       <c r="K420" t="inlineStr">
@@ -65656,7 +65656,7 @@
       <c r="I421" t="inlineStr"/>
       <c r="J421" t="inlineStr">
         <is>
-          <t>['France', 'Australia']</t>
+          <t>['Australia', 'France']</t>
         </is>
       </c>
       <c r="K421" t="inlineStr">
@@ -65968,7 +65968,7 @@
       </c>
       <c r="J423" t="inlineStr">
         <is>
-          <t>['France', 'Australia']</t>
+          <t>['Australia', 'France']</t>
         </is>
       </c>
       <c r="K423" t="inlineStr">
@@ -66266,7 +66266,7 @@
       </c>
       <c r="J425" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -66424,7 +66424,7 @@
       </c>
       <c r="J426" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K426" t="inlineStr">
@@ -66582,7 +66582,7 @@
       </c>
       <c r="J427" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K427" t="inlineStr">
@@ -66740,7 +66740,7 @@
       </c>
       <c r="J428" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
@@ -66898,7 +66898,7 @@
       </c>
       <c r="J429" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
@@ -67042,7 +67042,7 @@
       <c r="I430" t="inlineStr"/>
       <c r="J430" t="inlineStr">
         <is>
-          <t>['Morocco', 'Croatia']</t>
+          <t>['Croatia', 'Morocco']</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
@@ -67810,7 +67810,7 @@
       </c>
       <c r="J435" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany']</t>
+          <t>['Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
@@ -67968,7 +67968,7 @@
       </c>
       <c r="J436" t="inlineStr">
         <is>
-          <t>['Spain', 'Germany']</t>
+          <t>['Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K436" t="inlineStr">
@@ -68600,7 +68600,7 @@
       </c>
       <c r="J440" t="inlineStr">
         <is>
-          <t>['Japan', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Japan']</t>
         </is>
       </c>
       <c r="K440" t="inlineStr">
@@ -69530,7 +69530,7 @@
       </c>
       <c r="J446" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K446" t="inlineStr">
@@ -69688,7 +69688,7 @@
       </c>
       <c r="J447" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K447" t="inlineStr">
@@ -69846,7 +69846,7 @@
       </c>
       <c r="J448" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K448" t="inlineStr">
@@ -70004,7 +70004,7 @@
       </c>
       <c r="J449" t="inlineStr">
         <is>
-          <t>['Portugal', 'South Korea']</t>
+          <t>['South Korea', 'Portugal']</t>
         </is>
       </c>
       <c r="K449" t="inlineStr">
@@ -70148,7 +70148,7 @@
       <c r="I450" t="inlineStr"/>
       <c r="J450" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K450" t="inlineStr">
@@ -70302,7 +70302,7 @@
       </c>
       <c r="J451" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K451" t="inlineStr">
@@ -70460,7 +70460,7 @@
       </c>
       <c r="J452" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K452" t="inlineStr">
@@ -70776,7 +70776,7 @@
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K454" t="inlineStr">
@@ -70934,7 +70934,7 @@
       </c>
       <c r="J455" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K455" t="inlineStr">
@@ -71092,7 +71092,7 @@
       </c>
       <c r="J456" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K456" t="inlineStr">

</xml_diff>

<commit_message>
2nd and 4th contention
</commit_message>
<xml_diff>
--- a/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
+++ b/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
@@ -678,7 +678,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['Soviet Union', 'Hungary', 'France']</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>['Hungary', 'France', 'Soviet Union']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1608,7 +1608,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>['Italy', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Italy']</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2854,7 +2854,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Mexico', 'Belgium']</t>
+          <t>['Paraguay', 'Belgium', 'Mexico']</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -3784,7 +3784,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>['Portugal', 'Poland', 'Morocco']</t>
+          <t>['Morocco', 'Poland', 'Portugal']</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>['Portugal', 'Poland', 'England']</t>
+          <t>['England', 'Poland', 'Portugal']</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>['Portugal', 'England', 'Morocco']</t>
+          <t>['Morocco', 'England', 'Portugal']</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>['Morocco', 'Poland', 'England']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>['Morocco', 'Poland', 'England']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>['Morocco', 'Poland', 'England']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>['Morocco', 'Poland', 'England']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>['Morocco', 'Poland', 'England']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -5030,7 +5030,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Northern Ireland', 'Spain']</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>['Algeria', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Algeria', 'Spain']</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Northern Ireland', 'Spain']</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>['Algeria', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Algeria', 'Spain']</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Northern Ireland', 'Spain']</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Northern Ireland', 'Spain']</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Spain', 'Brazil']</t>
+          <t>['Brazil', 'Northern Ireland', 'Spain']</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -6574,7 +6574,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>['Romania', 'Argentina', 'Cameroon']</t>
+          <t>['Argentina', 'Romania', 'Cameroon']</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -8908,7 +8908,7 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -9694,7 +9694,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>['Italy', 'Austria', 'Czechoslovakia']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -9838,7 +9838,7 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Scotland', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>['Scotland', 'Sweden', 'Brazil']</t>
+          <t>['Brazil', 'Scotland', 'Sweden']</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Scotland', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Scotland', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Scotland', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -10610,7 +10610,7 @@
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Belgium', 'Spain']</t>
+          <t>['Belgium', 'Uruguay', 'Spain']</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Belgium', 'Spain']</t>
+          <t>['Belgium', 'Uruguay', 'Spain']</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Belgium', 'Spain']</t>
+          <t>['Belgium', 'Uruguay', 'Spain']</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Belgium', 'Spain']</t>
+          <t>['Belgium', 'Uruguay', 'Spain']</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Belgium', 'Spain']</t>
+          <t>['Belgium', 'Uruguay', 'Spain']</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -12150,7 +12150,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Romania', 'United States']</t>
+          <t>['Romania', 'United States', 'Switzerland']</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Romania', 'United States']</t>
+          <t>['Romania', 'United States', 'Switzerland']</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Romania', 'United States']</t>
+          <t>['Romania', 'United States', 'Switzerland']</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -12610,7 +12610,7 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -12922,7 +12922,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -13870,7 +13870,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'South Korea', 'Spain']</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -14172,7 +14172,7 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
-          <t>['Ireland', 'Mexico', 'Italy']</t>
+          <t>['Ireland', 'Italy', 'Mexico']</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>['Italy', 'Norway', 'Ireland']</t>
+          <t>['Ireland', 'Italy', 'Norway']</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>['Ireland', 'Mexico', 'Italy']</t>
+          <t>['Ireland', 'Italy', 'Mexico']</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -14628,7 +14628,7 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
-          <t>['Sweden', 'Cameroon', 'Brazil']</t>
+          <t>['Brazil', 'Sweden', 'Cameroon']</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -14782,7 +14782,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -15098,7 +15098,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -16046,7 +16046,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>['Sweden', 'Russia', 'Brazil']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -16190,7 +16190,7 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands', 'Saudi Arabia']</t>
+          <t>['Saudi Arabia', 'Belgium', 'Netherlands']</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -16344,7 +16344,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands', 'Saudi Arabia']</t>
+          <t>['Saudi Arabia', 'Belgium', 'Netherlands']</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -16502,7 +16502,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands', 'Saudi Arabia']</t>
+          <t>['Saudi Arabia', 'Belgium', 'Netherlands']</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -16660,7 +16660,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands', 'Saudi Arabia']</t>
+          <t>['Saudi Arabia', 'Belgium', 'Netherlands']</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -16818,7 +16818,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands', 'Saudi Arabia']</t>
+          <t>['Saudi Arabia', 'Belgium', 'Netherlands']</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -16962,7 +16962,7 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Nigeria']</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -17116,7 +17116,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Nigeria']</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -17274,7 +17274,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Nigeria']</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Nigeria']</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -17590,7 +17590,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
+          <t>['Argentina', 'Bulgaria', 'Nigeria']</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -17734,7 +17734,7 @@
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -17888,7 +17888,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -18046,7 +18046,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -18204,7 +18204,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -18362,7 +18362,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -18520,7 +18520,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>['Chile', 'Italy']</t>
+          <t>['Italy', 'Chile']</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -18664,7 +18664,7 @@
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
-          <t>['Norway', 'Brazil']</t>
+          <t>['Brazil', 'Norway']</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -18818,7 +18818,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>['Morocco', 'Brazil']</t>
+          <t>['Brazil', 'Morocco']</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>['Morocco', 'Brazil']</t>
+          <t>['Brazil', 'Morocco']</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -19134,7 +19134,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>['Morocco', 'Brazil']</t>
+          <t>['Brazil', 'Morocco']</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -19292,7 +19292,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>['Morocco', 'Brazil']</t>
+          <t>['Brazil', 'Morocco']</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -19450,7 +19450,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>['Morocco', 'Brazil']</t>
+          <t>['Brazil', 'Morocco']</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -19608,7 +19608,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>['Norway', 'Brazil']</t>
+          <t>['Brazil', 'Norway']</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -20998,7 +20998,7 @@
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -21152,7 +21152,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -21310,7 +21310,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -21942,7 +21942,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -22258,7 +22258,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -22416,7 +22416,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -22574,7 +22574,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -22732,7 +22732,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Paraguay']</t>
+          <t>['Paraguay', 'Nigeria']</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -24578,7 +24578,7 @@
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -24732,7 +24732,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -24890,7 +24890,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -25048,7 +25048,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -27526,7 +27526,7 @@
       <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Germany']</t>
+          <t>['Germany', 'Cameroon']</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -28456,7 +28456,7 @@
       <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -28610,7 +28610,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -28768,7 +28768,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -30474,7 +30474,7 @@
       <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -30628,7 +30628,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -30786,7 +30786,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -30944,7 +30944,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -31102,7 +31102,7 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -31260,7 +31260,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -31418,7 +31418,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -31576,7 +31576,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Brazil']</t>
+          <t>['Brazil', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -31734,7 +31734,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -31892,7 +31892,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -32050,7 +32050,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>['Turkey', 'Brazil']</t>
+          <t>['Brazil', 'Turkey']</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -33120,7 +33120,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -33594,7 +33594,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -33752,7 +33752,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -36072,7 +36072,7 @@
       <c r="I230" t="inlineStr"/>
       <c r="J230" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -36226,7 +36226,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -36384,7 +36384,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -36542,7 +36542,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -36700,7 +36700,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -36858,7 +36858,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -37016,7 +37016,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>['Sweden', 'England']</t>
+          <t>['England', 'Sweden']</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -37160,7 +37160,7 @@
       <c r="I237" t="inlineStr"/>
       <c r="J237" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -37314,7 +37314,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -37472,7 +37472,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -37630,7 +37630,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -37788,7 +37788,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -37946,7 +37946,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>['Portugal', 'Mexico']</t>
+          <t>['Mexico', 'Portugal']</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -39020,7 +39020,7 @@
       <c r="I249" t="inlineStr"/>
       <c r="J249" t="inlineStr">
         <is>
-          <t>['Italy', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Italy']</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -39174,7 +39174,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -39332,7 +39332,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -39490,7 +39490,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -39648,7 +39648,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -39806,7 +39806,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -39950,7 +39950,7 @@
       <c r="I255" t="inlineStr"/>
       <c r="J255" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -40104,7 +40104,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>['Croatia', 'Brazil']</t>
+          <t>['Brazil', 'Croatia']</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -40262,7 +40262,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>['Croatia', 'Brazil']</t>
+          <t>['Brazil', 'Croatia']</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -40420,7 +40420,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -40578,7 +40578,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -40736,7 +40736,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -40894,7 +40894,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>['Croatia', 'Brazil']</t>
+          <t>['Brazil', 'Croatia']</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -41052,7 +41052,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>['Croatia', 'Brazil']</t>
+          <t>['Brazil', 'Croatia']</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -41210,7 +41210,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -41368,7 +41368,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>['Australia', 'Brazil']</t>
+          <t>['Brazil', 'Australia']</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -41968,7 +41968,7 @@
       <c r="I268" t="inlineStr"/>
       <c r="J268" t="inlineStr">
         <is>
-          <t>['South Korea', 'Switzerland']</t>
+          <t>['Switzerland', 'South Korea']</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -42122,7 +42122,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>['South Korea', 'Switzerland']</t>
+          <t>['Switzerland', 'South Korea']</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -42740,7 +42740,7 @@
       <c r="I273" t="inlineStr"/>
       <c r="J273" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Mexico']</t>
+          <t>['Mexico', 'Uruguay']</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -42894,7 +42894,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Mexico']</t>
+          <t>['Mexico', 'Uruguay']</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -43052,7 +43052,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Mexico']</t>
+          <t>['Mexico', 'Uruguay']</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -43210,7 +43210,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Mexico']</t>
+          <t>['Mexico', 'Uruguay']</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -43368,7 +43368,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Mexico']</t>
+          <t>['Mexico', 'Uruguay']</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -43512,7 +43512,7 @@
       <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -43824,7 +43824,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -43982,7 +43982,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -44140,7 +44140,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -44298,7 +44298,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -44411,7 +44411,7 @@
         <v>0</v>
       </c>
       <c r="AR283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="284">
@@ -44456,7 +44456,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -44569,7 +44569,7 @@
         <v>0</v>
       </c>
       <c r="AR284" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="285">
@@ -44600,7 +44600,7 @@
       <c r="I285" t="inlineStr"/>
       <c r="J285" t="inlineStr">
         <is>
-          <t>['United States', 'Slovenia']</t>
+          <t>['Slovenia', 'United States']</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -44754,7 +44754,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>['England', 'Slovenia']</t>
+          <t>['Slovenia', 'England']</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -45056,7 +45056,7 @@
       <c r="I288" t="inlineStr"/>
       <c r="J288" t="inlineStr">
         <is>
-          <t>['Ghana', 'Germany']</t>
+          <t>['Germany', 'Ghana']</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -45210,7 +45210,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>['Ghana', 'Germany']</t>
+          <t>['Germany', 'Ghana']</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -45368,7 +45368,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>['Ghana', 'Germany']</t>
+          <t>['Germany', 'Ghana']</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -45526,7 +45526,7 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>['Ghana', 'Germany']</t>
+          <t>['Germany', 'Ghana']</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -45684,7 +45684,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>['Ghana', 'Germany']</t>
+          <t>['Germany', 'Ghana']</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -45797,7 +45797,7 @@
         <v>0</v>
       </c>
       <c r="AR292" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="293">
@@ -45828,7 +45828,7 @@
       <c r="I293" t="inlineStr"/>
       <c r="J293" t="inlineStr">
         <is>
-          <t>['Italy', 'Paraguay']</t>
+          <t>['Paraguay', 'Italy']</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -48004,7 +48004,7 @@
       <c r="I307" t="inlineStr"/>
       <c r="J307" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -48158,7 +48158,7 @@
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -48316,7 +48316,7 @@
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -48474,7 +48474,7 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -48618,7 +48618,7 @@
       <c r="I311" t="inlineStr"/>
       <c r="J311" t="inlineStr">
         <is>
-          <t>['Chile', 'Spain']</t>
+          <t>['Spain', 'Chile']</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -49232,7 +49232,7 @@
       <c r="I315" t="inlineStr"/>
       <c r="J315" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -49386,7 +49386,7 @@
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -49544,7 +49544,7 @@
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -49702,7 +49702,7 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -49860,7 +49860,7 @@
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -50018,7 +50018,7 @@
       </c>
       <c r="J320" t="inlineStr">
         <is>
-          <t>['Chile', 'Netherlands']</t>
+          <t>['Netherlands', 'Chile']</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
@@ -50162,7 +50162,7 @@
       <c r="I321" t="inlineStr"/>
       <c r="J321" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -50316,7 +50316,7 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
@@ -50474,7 +50474,7 @@
       </c>
       <c r="J323" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
@@ -50632,7 +50632,7 @@
       </c>
       <c r="J324" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K324" t="inlineStr">
@@ -50790,7 +50790,7 @@
       </c>
       <c r="J325" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K325" t="inlineStr">
@@ -50948,7 +50948,7 @@
       </c>
       <c r="J326" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K326" t="inlineStr">
@@ -51106,7 +51106,7 @@
       </c>
       <c r="J327" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
@@ -51264,7 +51264,7 @@
       </c>
       <c r="J328" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
@@ -51422,7 +51422,7 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -51580,7 +51580,7 @@
       </c>
       <c r="J330" t="inlineStr">
         <is>
-          <t>['Mexico', 'Brazil']</t>
+          <t>['Brazil', 'Mexico']</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
@@ -51724,7 +51724,7 @@
       <c r="I331" t="inlineStr"/>
       <c r="J331" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Italy']</t>
+          <t>['Italy', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
@@ -53426,7 +53426,7 @@
       <c r="I342" t="inlineStr"/>
       <c r="J342" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
@@ -53580,7 +53580,7 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
@@ -53738,7 +53738,7 @@
       </c>
       <c r="J344" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
@@ -53896,7 +53896,7 @@
       </c>
       <c r="J345" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K345" t="inlineStr">
@@ -54054,7 +54054,7 @@
       </c>
       <c r="J346" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K346" t="inlineStr">
@@ -54212,7 +54212,7 @@
       </c>
       <c r="J347" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
@@ -54370,7 +54370,7 @@
       </c>
       <c r="J348" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K348" t="inlineStr">
@@ -54528,7 +54528,7 @@
       </c>
       <c r="J349" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K349" t="inlineStr">
@@ -54686,7 +54686,7 @@
       </c>
       <c r="J350" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K350" t="inlineStr">
@@ -54844,7 +54844,7 @@
       </c>
       <c r="J351" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Argentina']</t>
+          <t>['Argentina', 'Nigeria']</t>
         </is>
       </c>
       <c r="K351" t="inlineStr">
@@ -56374,7 +56374,7 @@
       <c r="I361" t="inlineStr"/>
       <c r="J361" t="inlineStr">
         <is>
-          <t>['Algeria', 'Belgium']</t>
+          <t>['Belgium', 'Algeria']</t>
         </is>
       </c>
       <c r="K361" t="inlineStr">
@@ -56686,7 +56686,7 @@
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>['Algeria', 'Belgium']</t>
+          <t>['Belgium', 'Algeria']</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
@@ -56844,7 +56844,7 @@
       </c>
       <c r="J364" t="inlineStr">
         <is>
-          <t>['Algeria', 'Belgium']</t>
+          <t>['Belgium', 'Algeria']</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
@@ -56988,7 +56988,7 @@
       <c r="I365" t="inlineStr"/>
       <c r="J365" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
@@ -57142,7 +57142,7 @@
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
@@ -57300,7 +57300,7 @@
       </c>
       <c r="J367" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K367" t="inlineStr">
@@ -57458,7 +57458,7 @@
       </c>
       <c r="J368" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K368" t="inlineStr">
@@ -57616,7 +57616,7 @@
       </c>
       <c r="J369" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K369" t="inlineStr">
@@ -57774,7 +57774,7 @@
       </c>
       <c r="J370" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K370" t="inlineStr">
@@ -57932,7 +57932,7 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>['Uruguay', 'Russia']</t>
+          <t>['Russia', 'Uruguay']</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -59774,7 +59774,7 @@
       </c>
       <c r="J383" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
@@ -60406,7 +60406,7 @@
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
@@ -60564,7 +60564,7 @@
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
@@ -60708,7 +60708,7 @@
       <c r="I389" t="inlineStr"/>
       <c r="J389" t="inlineStr">
         <is>
-          <t>['Mexico', 'Germany']</t>
+          <t>['Germany', 'Mexico']</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
@@ -61638,7 +61638,7 @@
       <c r="I395" t="inlineStr"/>
       <c r="J395" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
@@ -61792,7 +61792,7 @@
       </c>
       <c r="J396" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
@@ -61950,7 +61950,7 @@
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
@@ -62108,7 +62108,7 @@
       </c>
       <c r="J398" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
@@ -62266,7 +62266,7 @@
       </c>
       <c r="J399" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
@@ -62424,7 +62424,7 @@
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
@@ -62582,7 +62582,7 @@
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
@@ -63182,7 +63182,7 @@
       <c r="I405" t="inlineStr"/>
       <c r="J405" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
@@ -63336,7 +63336,7 @@
       </c>
       <c r="J406" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
@@ -63494,7 +63494,7 @@
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
@@ -63652,7 +63652,7 @@
       </c>
       <c r="J408" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
@@ -63810,7 +63810,7 @@
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
@@ -65810,7 +65810,7 @@
       </c>
       <c r="J422" t="inlineStr">
         <is>
-          <t>['France', 'Tunisia']</t>
+          <t>['Tunisia', 'France']</t>
         </is>
       </c>
       <c r="K422" t="inlineStr">
@@ -67196,7 +67196,7 @@
       </c>
       <c r="J431" t="inlineStr">
         <is>
-          <t>['Morocco', 'Croatia']</t>
+          <t>['Croatia', 'Morocco']</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
@@ -67354,7 +67354,7 @@
       </c>
       <c r="J432" t="inlineStr">
         <is>
-          <t>['Morocco', 'Croatia']</t>
+          <t>['Croatia', 'Morocco']</t>
         </is>
       </c>
       <c r="K432" t="inlineStr">
@@ -67512,7 +67512,7 @@
       </c>
       <c r="J433" t="inlineStr">
         <is>
-          <t>['Morocco', 'Croatia']</t>
+          <t>['Croatia', 'Morocco']</t>
         </is>
       </c>
       <c r="K433" t="inlineStr">
@@ -68600,7 +68600,7 @@
       </c>
       <c r="J440" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Japan']</t>
+          <t>['Japan', 'Costa Rica']</t>
         </is>
       </c>
       <c r="K440" t="inlineStr">
@@ -69218,7 +69218,7 @@
       <c r="I444" t="inlineStr"/>
       <c r="J444" t="inlineStr">
         <is>
-          <t>['Portugal', 'Ghana']</t>
+          <t>['Ghana', 'Portugal']</t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
@@ -69372,7 +69372,7 @@
       </c>
       <c r="J445" t="inlineStr">
         <is>
-          <t>['Portugal', 'Ghana']</t>
+          <t>['Ghana', 'Portugal']</t>
         </is>
       </c>
       <c r="K445" t="inlineStr">
@@ -70148,7 +70148,7 @@
       <c r="I450" t="inlineStr"/>
       <c r="J450" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K450" t="inlineStr">
@@ -70302,7 +70302,7 @@
       </c>
       <c r="J451" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K451" t="inlineStr">
@@ -70460,7 +70460,7 @@
       </c>
       <c r="J452" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K452" t="inlineStr">
@@ -70618,7 +70618,7 @@
       </c>
       <c r="J453" t="inlineStr">
         <is>
-          <t>['Serbia', 'Brazil']</t>
+          <t>['Brazil', 'Serbia']</t>
         </is>
       </c>
       <c r="K453" t="inlineStr">
@@ -70776,7 +70776,7 @@
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K454" t="inlineStr">
@@ -70934,7 +70934,7 @@
       </c>
       <c r="J455" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K455" t="inlineStr">
@@ -71092,7 +71092,7 @@
       </c>
       <c r="J456" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Brazil']</t>
+          <t>['Brazil', 'Switzerland']</t>
         </is>
       </c>
       <c r="K456" t="inlineStr">

</xml_diff>

<commit_message>
2nd and 4th wc uefa
</commit_message>
<xml_diff>
--- a/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
+++ b/data/out/wiki/men/fifa/wc/goals_wc_fifa.xlsx
@@ -678,7 +678,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>['Soviet Union', 'Hungary', 'France']</t>
+          <t>['France', 'Hungary', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1608,7 +1608,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Argentina', 'Italy', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>['Italy', 'Bulgaria', 'Argentina']</t>
+          <t>['Bulgaria', 'Argentina', 'Italy']</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>['Belgium', 'Paraguay', 'Mexico']</t>
+          <t>['Mexico', 'Paraguay', 'Belgium']</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>['Mexico', 'Belgium', 'Paraguay']</t>
+          <t>['Mexico', 'Paraguay', 'Belgium']</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3784,7 +3784,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>['Portugal', 'Poland', 'Morocco']</t>
+          <t>['Morocco', 'Portugal', 'Poland']</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Portugal']</t>
+          <t>['England', 'Portugal', 'Poland']</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>['England', 'Portugal', 'Morocco']</t>
+          <t>['Morocco', 'England', 'Portugal']</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Morocco']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Morocco']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Morocco']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Morocco']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>['England', 'Poland', 'Morocco']</t>
+          <t>['England', 'Morocco', 'Poland']</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -5030,7 +5030,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Brazil', 'Northern Ireland']</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>['Algeria', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Algeria', 'Brazil']</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Brazil', 'Northern Ireland']</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>['Algeria', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Algeria', 'Brazil']</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Brazil', 'Northern Ireland']</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Brazil', 'Northern Ireland']</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>['Northern Ireland', 'Brazil', 'Spain']</t>
+          <t>['Spain', 'Brazil', 'Northern Ireland']</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -6118,7 +6118,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>['West Germany', 'Uruguay', 'Denmark']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>['West Germany', 'Uruguay', 'Denmark']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>['West Germany', 'Uruguay', 'Denmark']</t>
+          <t>['West Germany', 'Denmark', 'Uruguay']</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -6574,7 +6574,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Soviet Union', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Soviet Union']</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>['Cameroon', 'Romania', 'Argentina']</t>
+          <t>['Cameroon', 'Argentina', 'Romania']</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -7974,7 +7974,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -8448,7 +8448,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'West Germany', 'Colombia']</t>
+          <t>['West Germany', 'Colombia', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -8908,7 +8908,7 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -9694,7 +9694,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>['Czechoslovakia', 'Italy', 'Austria']</t>
+          <t>['Czechoslovakia', 'Austria', 'Italy']</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -9838,7 +9838,7 @@
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>['Costa Rica', 'Scotland', 'Brazil']</t>
+          <t>['Costa Rica', 'Brazil', 'Scotland']</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>['Scotland', 'Brazil', 'Sweden']</t>
+          <t>['Sweden', 'Brazil', 'Scotland']</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Costa Rica', 'Brazil', 'Scotland']</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Costa Rica', 'Brazil', 'Scotland']</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>['Scotland', 'Costa Rica', 'Brazil']</t>
+          <t>['Costa Rica', 'Brazil', 'Scotland']</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -10610,7 +10610,7 @@
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
-          <t>['Belgium', 'Uruguay', 'Spain']</t>
+          <t>['Uruguay', 'Spain', 'Belgium']</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>['Belgium', 'Uruguay', 'Spain']</t>
+          <t>['Uruguay', 'Spain', 'Belgium']</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>['Belgium', 'Uruguay', 'Spain']</t>
+          <t>['Uruguay', 'Spain', 'Belgium']</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>['Belgium', 'Uruguay', 'Spain']</t>
+          <t>['Uruguay', 'Spain', 'Belgium']</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>['Belgium', 'Uruguay', 'Spain']</t>
+          <t>['Uruguay', 'Spain', 'Belgium']</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -11382,7 +11382,7 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>['Ireland', 'England', 'Netherlands']</t>
+          <t>['Netherlands', 'England', 'Ireland']</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>['England', 'Netherlands', 'Egypt']</t>
+          <t>['Egypt', 'Netherlands', 'England']</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>['England', 'Netherlands', 'Egypt']</t>
+          <t>['Egypt', 'Netherlands', 'England']</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>['Ireland', 'England', 'Netherlands']</t>
+          <t>['Netherlands', 'England', 'Ireland']</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -11996,7 +11996,7 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['United States', 'Switzerland', 'Romania']</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -12150,7 +12150,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['United States', 'Switzerland', 'Romania']</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['United States', 'Switzerland', 'Romania']</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>['United States', 'Romania', 'Switzerland']</t>
+          <t>['United States', 'Switzerland', 'Romania']</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -12610,7 +12610,7 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -12922,7 +12922,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -13870,7 +13870,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>['South Korea', 'Germany', 'Spain']</t>
+          <t>['Germany', 'Spain', 'South Korea']</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -14172,7 +14172,7 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
-          <t>['Ireland', 'Mexico', 'Italy']</t>
+          <t>['Mexico', 'Ireland', 'Italy']</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>['Ireland', 'Norway', 'Italy']</t>
+          <t>['Norway', 'Ireland', 'Italy']</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>['Ireland', 'Mexico', 'Italy']</t>
+          <t>['Mexico', 'Ireland', 'Italy']</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -14782,7 +14782,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Sweden', 'Russia']</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -15098,7 +15098,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Sweden', 'Russia']</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Sweden', 'Russia']</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Sweden', 'Russia']</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -15888,7 +15888,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -16046,7 +16046,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>['Russia', 'Brazil', 'Sweden']</t>
+          <t>['Brazil', 'Russia', 'Sweden']</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -16190,7 +16190,7 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
-          <t>['Belgium', 'Saudi Arabia', 'Netherlands']</t>
+          <t>['Saudi Arabia', 'Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -16344,7 +16344,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>['Belgium', 'Saudi Arabia', 'Netherlands']</t>
+          <t>['Saudi Arabia', 'Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -16502,7 +16502,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>['Belgium', 'Saudi Arabia', 'Netherlands']</t>
+          <t>['Saudi Arabia', 'Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -16660,7 +16660,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>['Belgium', 'Saudi Arabia', 'Netherlands']</t>
+          <t>['Saudi Arabia', 'Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -16818,7 +16818,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>['Belgium', 'Saudi Arabia', 'Netherlands']</t>
+          <t>['Saudi Arabia', 'Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -16962,7 +16962,7 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Bulgaria', 'Argentina']</t>
+          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -17116,7 +17116,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Bulgaria', 'Argentina']</t>
+          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -17274,7 +17274,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Bulgaria', 'Argentina']</t>
+          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Bulgaria', 'Argentina']</t>
+          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -17590,7 +17590,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>['Nigeria', 'Bulgaria', 'Argentina']</t>
+          <t>['Nigeria', 'Argentina', 'Bulgaria']</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -18818,7 +18818,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>['Brazil', 'Morocco']</t>
+          <t>['Morocco', 'Brazil']</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>['Brazil', 'Morocco']</t>
+          <t>['Morocco', 'Brazil']</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -19134,7 +19134,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>['Brazil', 'Morocco']</t>
+          <t>['Morocco', 'Brazil']</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -19292,7 +19292,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>['Brazil', 'Morocco']</t>
+          <t>['Morocco', 'Brazil']</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -19450,7 +19450,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>['Brazil', 'Morocco']</t>
+          <t>['Morocco', 'Brazil']</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -19752,7 +19752,7 @@
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -19906,7 +19906,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -20064,7 +20064,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -20222,7 +20222,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -20380,7 +20380,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -20696,7 +20696,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -20854,7 +20854,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -22876,7 +22876,7 @@
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr">
         <is>
-          <t>['Mexico', 'Netherlands']</t>
+          <t>['Netherlands', 'Mexico']</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -23030,7 +23030,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>['Mexico', 'Netherlands']</t>
+          <t>['Netherlands', 'Mexico']</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -23188,7 +23188,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands']</t>
+          <t>['Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -23346,7 +23346,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>['Belgium', 'Netherlands']</t>
+          <t>['Netherlands', 'Belgium']</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -23504,7 +23504,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>['Mexico', 'Netherlands']</t>
+          <t>['Netherlands', 'Mexico']</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -23662,7 +23662,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>['Mexico', 'Netherlands']</t>
+          <t>['Netherlands', 'Mexico']</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -23820,7 +23820,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>['Mexico', 'Netherlands']</t>
+          <t>['Netherlands', 'Mexico']</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -23964,7 +23964,7 @@
       <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Germany']</t>
+          <t>['Germany', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -24118,7 +24118,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Germany']</t>
+          <t>['Germany', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -24276,7 +24276,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Germany']</t>
+          <t>['Germany', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -24434,7 +24434,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Germany']</t>
+          <t>['Germany', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -24578,7 +24578,7 @@
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -24732,7 +24732,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -24890,7 +24890,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -25048,7 +25048,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -26122,7 +26122,7 @@
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -26276,7 +26276,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -26389,7 +26389,7 @@
         <v>1</v>
       </c>
       <c r="AR167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -26434,7 +26434,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -26592,7 +26592,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -26750,7 +26750,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -26908,7 +26908,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -27066,7 +27066,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -27224,7 +27224,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>['Senegal', 'Denmark']</t>
+          <t>['Denmark', 'Senegal']</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -27680,7 +27680,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>['Ireland', 'Germany']</t>
+          <t>['Germany', 'Ireland']</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -27838,7 +27838,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>['Ireland', 'Germany']</t>
+          <t>['Germany', 'Ireland']</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -27996,7 +27996,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>['Ireland', 'Germany']</t>
+          <t>['Germany', 'Ireland']</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -28154,7 +28154,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>['Ireland', 'Germany']</t>
+          <t>['Germany', 'Ireland']</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -28312,7 +28312,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>['Ireland', 'Germany']</t>
+          <t>['Germany', 'Ireland']</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -28912,7 +28912,7 @@
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -29066,7 +29066,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -29224,7 +29224,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -29382,7 +29382,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -29540,7 +29540,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -29698,7 +29698,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -29856,7 +29856,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -30014,7 +30014,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -30172,7 +30172,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>['Spain', 'South Africa']</t>
+          <t>['South Africa', 'Spain']</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -30330,7 +30330,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Spain']</t>
+          <t>['Spain', 'Paraguay']</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -32808,7 +32808,7 @@
       <c r="I209" t="inlineStr"/>
       <c r="J209" t="inlineStr">
         <is>
-          <t>['Russia', 'Japan']</t>
+          <t>['Japan', 'Russia']</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -33120,7 +33120,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -33278,7 +33278,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>['Russia', 'Japan']</t>
+          <t>['Japan', 'Russia']</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -33436,7 +33436,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>['Russia', 'Japan']</t>
+          <t>['Japan', 'Russia']</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -33594,7 +33594,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -33752,7 +33752,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>['Belgium', 'Japan']</t>
+          <t>['Japan', 'Belgium']</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -34208,7 +34208,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>['South Korea', 'Portugal']</t>
+          <t>['Portugal', 'South Korea']</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -34366,7 +34366,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>['South Korea', 'Portugal']</t>
+          <t>['Portugal', 'South Korea']</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>['South Korea', 'Portugal']</t>
+          <t>['Portugal', 'South Korea']</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -38090,7 +38090,7 @@
       <c r="I243" t="inlineStr"/>
       <c r="J243" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -38244,7 +38244,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -38402,7 +38402,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -38560,7 +38560,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -38718,7 +38718,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -38876,7 +38876,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Argentina']</t>
+          <t>['Argentina', 'Netherlands']</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -39020,7 +39020,7 @@
       <c r="I249" t="inlineStr"/>
       <c r="J249" t="inlineStr">
         <is>
-          <t>['Italy', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Italy']</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -39174,7 +39174,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -39332,7 +39332,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -39490,7 +39490,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -39648,7 +39648,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -39806,7 +39806,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>['Italy', 'Ghana']</t>
+          <t>['Ghana', 'Italy']</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -41968,7 +41968,7 @@
       <c r="I268" t="inlineStr"/>
       <c r="J268" t="inlineStr">
         <is>
-          <t>['South Korea', 'Switzerland']</t>
+          <t>['Switzerland', 'South Korea']</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -42122,7 +42122,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>['South Korea', 'Switzerland']</t>
+          <t>['Switzerland', 'South Korea']</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -42280,7 +42280,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -42438,7 +42438,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -42596,7 +42596,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -42740,7 +42740,7 @@
       <c r="I273" t="inlineStr"/>
       <c r="J273" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -42894,7 +42894,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -43052,7 +43052,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -43210,7 +43210,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -43368,7 +43368,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>['Mexico', 'Uruguay']</t>
+          <t>['Uruguay', 'Mexico']</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -43512,7 +43512,7 @@
       <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -43824,7 +43824,7 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -43982,7 +43982,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -44140,7 +44140,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -44298,7 +44298,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -44456,7 +44456,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>['South Korea', 'Argentina']</t>
+          <t>['Argentina', 'South Korea']</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -44600,7 +44600,7 @@
       <c r="I285" t="inlineStr"/>
       <c r="J285" t="inlineStr">
         <is>
-          <t>['Slovenia', 'United States']</t>
+          <t>['United States', 'Slovenia']</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -44754,7 +44754,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>['Slovenia', 'England']</t>
+          <t>['England', 'Slovenia']</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -45056,7 +45056,7 @@
       <c r="I288" t="inlineStr"/>
       <c r="J288" t="inlineStr">
         <is>
-          <t>['Germany', 'Ghana']</t>
+          <t>['Ghana', 'Germany']</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -45210,7 +45210,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>['Germany', 'Ghana']</t>
+          <t>['Ghana', 'Germany']</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -45368,7 +45368,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>['Germany', 'Ghana']</t>
+          <t>['Ghana', 'Germany']</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -45526,7 +45526,7 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>['Germany', 'Ghana']</t>
+          <t>['Ghana', 'Germany']</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -45684,7 +45684,7 @@
       </c>
       <c r="J292" t="inlineStr">
         <is>
-          <t>['Germany', 'Ghana']</t>
+          <t>['Ghana', 'Germany']</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -45982,7 +45982,7 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Slovakia']</t>
+          <t>['Slovakia', 'Paraguay']</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -46140,7 +46140,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Slovakia']</t>
+          <t>['Slovakia', 'Paraguay']</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -46298,7 +46298,7 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Slovakia']</t>
+          <t>['Slovakia', 'Paraguay']</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -46456,7 +46456,7 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Slovakia']</t>
+          <t>['Slovakia', 'Paraguay']</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
@@ -46614,7 +46614,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>['Paraguay', 'Slovakia']</t>
+          <t>['Slovakia', 'Paraguay']</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -46758,7 +46758,7 @@
       <c r="I299" t="inlineStr"/>
       <c r="J299" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -46912,7 +46912,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -47070,7 +47070,7 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -47228,7 +47228,7 @@
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -47386,7 +47386,7 @@
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
@@ -47544,7 +47544,7 @@
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
@@ -47702,7 +47702,7 @@
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
@@ -47860,7 +47860,7 @@
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>['Japan', 'Netherlands']</t>
+          <t>['Netherlands', 'Japan']</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -48004,7 +48004,7 @@
       <c r="I307" t="inlineStr"/>
       <c r="J307" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -48158,7 +48158,7 @@
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -48316,7 +48316,7 @@
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -48474,7 +48474,7 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>['Portugal', 'Brazil']</t>
+          <t>['Brazil', 'Portugal']</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -51724,7 +51724,7 @@
       <c r="I331" t="inlineStr"/>
       <c r="J331" t="inlineStr">
         <is>
-          <t>['Italy', 'Costa Rica']</t>
+          <t>['Costa Rica', 'Italy']</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
@@ -52334,7 +52334,7 @@
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
@@ -52492,7 +52492,7 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
@@ -52650,7 +52650,7 @@
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
@@ -53282,7 +53282,7 @@
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>['Colombia', 'Greece']</t>
+          <t>['Greece', 'Colombia']</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -54988,7 +54988,7 @@
       <c r="I352" t="inlineStr"/>
       <c r="J352" t="inlineStr">
         <is>
-          <t>['Ecuador', 'France']</t>
+          <t>['France', 'Ecuador']</t>
         </is>
       </c>
       <c r="K352" t="inlineStr">
@@ -55142,7 +55142,7 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
@@ -55300,7 +55300,7 @@
       </c>
       <c r="J354" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K354" t="inlineStr">
@@ -55458,7 +55458,7 @@
       </c>
       <c r="J355" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France']</t>
+          <t>['France', 'Switzerland']</t>
         </is>
       </c>
       <c r="K355" t="inlineStr">
@@ -56528,7 +56528,7 @@
       </c>
       <c r="J362" t="inlineStr">
         <is>
-          <t>['Belgium', 'Russia']</t>
+          <t>['Russia', 'Belgium']</t>
         </is>
       </c>
       <c r="K362" t="inlineStr">
@@ -56988,7 +56988,7 @@
       <c r="I365" t="inlineStr"/>
       <c r="J365" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K365" t="inlineStr">
@@ -57142,7 +57142,7 @@
       </c>
       <c r="J366" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K366" t="inlineStr">
@@ -57300,7 +57300,7 @@
       </c>
       <c r="J367" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K367" t="inlineStr">
@@ -57458,7 +57458,7 @@
       </c>
       <c r="J368" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K368" t="inlineStr">
@@ -57616,7 +57616,7 @@
       </c>
       <c r="J369" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K369" t="inlineStr">
@@ -57774,7 +57774,7 @@
       </c>
       <c r="J370" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K370" t="inlineStr">
@@ -57932,7 +57932,7 @@
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>['Russia', 'Uruguay']</t>
+          <t>['Uruguay', 'Russia']</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -58076,7 +58076,7 @@
       <c r="I372" t="inlineStr"/>
       <c r="J372" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K372" t="inlineStr">
@@ -58230,7 +58230,7 @@
       </c>
       <c r="J373" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K373" t="inlineStr">
@@ -58388,7 +58388,7 @@
       </c>
       <c r="J374" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K374" t="inlineStr">
@@ -58546,7 +58546,7 @@
       </c>
       <c r="J375" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K375" t="inlineStr">
@@ -58704,7 +58704,7 @@
       </c>
       <c r="J376" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K376" t="inlineStr">
@@ -58862,7 +58862,7 @@
       </c>
       <c r="J377" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K377" t="inlineStr">
@@ -59020,7 +59020,7 @@
       </c>
       <c r="J378" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K378" t="inlineStr">
@@ -59164,7 +59164,7 @@
       <c r="I379" t="inlineStr"/>
       <c r="J379" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K379" t="inlineStr">
@@ -59318,7 +59318,7 @@
       </c>
       <c r="J380" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K380" t="inlineStr">
@@ -59476,7 +59476,7 @@
       </c>
       <c r="J381" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K381" t="inlineStr">
@@ -59620,7 +59620,7 @@
       <c r="I382" t="inlineStr"/>
       <c r="J382" t="inlineStr">
         <is>
-          <t>['Croatia', 'Nigeria']</t>
+          <t>['Nigeria', 'Croatia']</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
@@ -59774,7 +59774,7 @@
       </c>
       <c r="J383" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
@@ -59932,7 +59932,7 @@
       </c>
       <c r="J384" t="inlineStr">
         <is>
-          <t>['Croatia', 'Nigeria']</t>
+          <t>['Nigeria', 'Croatia']</t>
         </is>
       </c>
       <c r="K384" t="inlineStr">
@@ -60090,7 +60090,7 @@
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>['Croatia', 'Nigeria']</t>
+          <t>['Nigeria', 'Croatia']</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
@@ -60248,7 +60248,7 @@
       </c>
       <c r="J386" t="inlineStr">
         <is>
-          <t>['Croatia', 'Nigeria']</t>
+          <t>['Nigeria', 'Croatia']</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
@@ -60406,7 +60406,7 @@
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
@@ -60564,7 +60564,7 @@
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>['Croatia', 'Argentina']</t>
+          <t>['Argentina', 'Croatia']</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
@@ -60708,7 +60708,7 @@
       <c r="I389" t="inlineStr"/>
       <c r="J389" t="inlineStr">
         <is>
-          <t>['Mexico', 'Germany']</t>
+          <t>['Germany', 'Mexico']</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
@@ -61638,7 +61638,7 @@
       <c r="I395" t="inlineStr"/>
       <c r="J395" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
@@ -61792,7 +61792,7 @@
       </c>
       <c r="J396" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
@@ -61950,7 +61950,7 @@
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
@@ -62108,7 +62108,7 @@
       </c>
       <c r="J398" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
@@ -62266,7 +62266,7 @@
       </c>
       <c r="J399" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
@@ -62424,7 +62424,7 @@
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
@@ -62582,7 +62582,7 @@
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
@@ -62880,7 +62880,7 @@
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>['Colombia', 'Senegal']</t>
+          <t>['Senegal', 'Colombia']</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
@@ -63038,7 +63038,7 @@
       </c>
       <c r="J404" t="inlineStr">
         <is>
-          <t>['Colombia', 'Senegal']</t>
+          <t>['Senegal', 'Colombia']</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
@@ -63182,7 +63182,7 @@
       <c r="I405" t="inlineStr"/>
       <c r="J405" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
@@ -63336,7 +63336,7 @@
       </c>
       <c r="J406" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
@@ -63494,7 +63494,7 @@
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
@@ -63652,7 +63652,7 @@
       </c>
       <c r="J408" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
@@ -63810,7 +63810,7 @@
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>['Belgium', 'England']</t>
+          <t>['England', 'Belgium']</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
@@ -65656,7 +65656,7 @@
       <c r="I421" t="inlineStr"/>
       <c r="J421" t="inlineStr">
         <is>
-          <t>['Australia', 'France']</t>
+          <t>['France', 'Australia']</t>
         </is>
       </c>
       <c r="K421" t="inlineStr">
@@ -65810,7 +65810,7 @@
       </c>
       <c r="J422" t="inlineStr">
         <is>
-          <t>['Tunisia', 'France']</t>
+          <t>['France', 'Tunisia']</t>
         </is>
       </c>
       <c r="K422" t="inlineStr">
@@ -65968,7 +65968,7 @@
       </c>
       <c r="J423" t="inlineStr">
         <is>
-          <t>['Australia', 'France']</t>
+          <t>['France', 'Australia']</t>
         </is>
       </c>
       <c r="K423" t="inlineStr">
@@ -66112,7 +66112,7 @@
       <c r="I424" t="inlineStr"/>
       <c r="J424" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
@@ -66266,7 +66266,7 @@
       </c>
       <c r="J425" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -66424,7 +66424,7 @@
       </c>
       <c r="J426" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K426" t="inlineStr">
@@ -66582,7 +66582,7 @@
       </c>
       <c r="J427" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K427" t="inlineStr">
@@ -66740,7 +66740,7 @@
       </c>
       <c r="J428" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
@@ -66898,7 +66898,7 @@
       </c>
       <c r="J429" t="inlineStr">
         <is>
-          <t>['Poland', 'Argentina']</t>
+          <t>['Argentina', 'Poland']</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
@@ -67042,7 +67042,7 @@
       <c r="I430" t="inlineStr"/>
       <c r="J430" t="inlineStr">
         <is>
-          <t>['Croatia', 'Morocco']</t>
+          <t>['Morocco', 'Croatia']</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
@@ -67196,7 +67196,7 @@
       </c>
       <c r="J431" t="inlineStr">
         <is>
-          <t>['Croatia', 'Morocco']</t>
+          <t>['Morocco', 'Croatia']</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
@@ -67354,7 +67354,7 @@
       </c>
       <c r="J432" t="inlineStr">
         <is>
-          <t>['Croatia', 'Morocco']</t>
+          <t>['Morocco', 'Croatia']</t>
         </is>
       </c>
       <c r="K432" t="inlineStr">
@@ -67512,7 +67512,7 @@
       </c>
       <c r="J433" t="inlineStr">
         <is>
-          <t>['Croatia', 'Morocco']</t>
+          <t>['Morocco', 'Croatia']</t>
         </is>
       </c>
       <c r="K433" t="inlineStr">
@@ -69218,7 +69218,7 @@
       <c r="I444" t="inlineStr"/>
       <c r="J444" t="inlineStr">
         <is>
-          <t>['Portugal', 'Ghana']</t>
+          <t>['Ghana', 'Portugal']</t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
@@ -69372,7 +69372,7 @@
       </c>
       <c r="J445" t="inlineStr">
         <is>
-          <t>['Portugal', 'Ghana']</t>
+          <t>['Ghana', 'Portugal']</t>
         </is>
       </c>
       <c r="K445" t="inlineStr">
@@ -69530,7 +69530,7 @@
       </c>
       <c r="J446" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K446" t="inlineStr">
@@ -69688,7 +69688,7 @@
       </c>
       <c r="J447" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K447" t="inlineStr">
@@ -69846,7 +69846,7 @@
       </c>
       <c r="J448" t="inlineStr">
         <is>
-          <t>['Portugal', 'Uruguay']</t>
+          <t>['Uruguay', 'Portugal']</t>
         </is>
       </c>
       <c r="K448" t="inlineStr">
@@ -70148,7 +70148,7 @@
       <c r="I450" t="inlineStr"/>
       <c r="J450" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K450" t="inlineStr">
@@ -70302,7 +70302,7 @@
       </c>
       <c r="J451" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K451" t="inlineStr">
@@ -70460,7 +70460,7 @@
       </c>
       <c r="J452" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K452" t="inlineStr">
@@ -70776,7 +70776,7 @@
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K454" t="inlineStr">
@@ -70934,7 +70934,7 @@
       </c>
       <c r="J455" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K455" t="inlineStr">
@@ -71092,7 +71092,7 @@
       </c>
       <c r="J456" t="inlineStr">
         <is>
-          <t>['Brazil', 'Switzerland']</t>
+          <t>['Switzerland', 'Brazil']</t>
         </is>
       </c>
       <c r="K456" t="inlineStr">

</xml_diff>